<commit_message>
Daily slate 2026-04-30 [auto]
</commit_message>
<xml_diff>
--- a/NBA/step8_nba1q_direction_clean.xlsx
+++ b/NBA/step8_nba1q_direction_clean.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ211"/>
+  <dimension ref="A1:BJ212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -37502,7 +37502,7 @@
         </is>
       </c>
       <c r="B171" s="5" t="n">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="C171" s="5" t="inlineStr">
         <is>
@@ -43274,24 +43274,24 @@
       <c r="B207" s="5" t="inlineStr"/>
       <c r="C207" s="5" t="inlineStr">
         <is>
-          <t>Tim Hardaway</t>
+          <t>Rudy Gobert</t>
         </is>
       </c>
       <c r="D207" s="5" t="inlineStr">
         <is>
-          <t>G-F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E207" s="5" t="inlineStr">
         <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="F207" s="5" t="inlineStr">
+        <is>
           <t>DEN</t>
         </is>
       </c>
-      <c r="F207" s="5" t="inlineStr">
-        <is>
-          <t>MIN</t>
-        </is>
-      </c>
       <c r="G207" s="5" t="inlineStr">
         <is>
           <t>2026-04-30 21:30:00-04:00</t>
@@ -43317,30 +43317,46 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="L207" s="5" t="inlineStr"/>
-      <c r="M207" s="5" t="inlineStr"/>
+      <c r="L207" s="5" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="M207" s="5" t="n">
+        <v>0.2</v>
+      </c>
       <c r="N207" s="5" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="O207" s="5" t="n">
-        <v>0.8335</v>
+        <v>0.8636</v>
       </c>
       <c r="P207" s="5" t="inlineStr"/>
       <c r="Q207" s="5" t="inlineStr"/>
-      <c r="R207" s="5" t="inlineStr"/>
-      <c r="S207" s="5" t="inlineStr"/>
-      <c r="T207" s="5" t="inlineStr"/>
-      <c r="U207" s="5" t="inlineStr"/>
-      <c r="V207" s="5" t="inlineStr"/>
-      <c r="W207" s="5" t="inlineStr"/>
+      <c r="R207" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="S207" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="T207" s="5" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="U207" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="V207" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="W207" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="X207" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>21</t>
         </is>
       </c>
       <c r="Y207" s="5" t="inlineStr">
         <is>
-          <t>Above Avg</t>
+          <t>Avg</t>
         </is>
       </c>
       <c r="Z207" s="5" t="inlineStr">
@@ -43355,34 +43371,90 @@
       </c>
       <c r="AB207" s="5" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="AC207" s="5" t="inlineStr">
-        <is>
-          <t>NO_PROJECTION_OR_LINE</t>
-        </is>
-      </c>
-      <c r="AD207" s="5" t="inlineStr"/>
-      <c r="AE207" s="5" t="inlineStr"/>
-      <c r="AF207" s="5" t="inlineStr"/>
+          <t>SUPPORT</t>
+        </is>
+      </c>
+      <c r="AC207" s="5" t="inlineStr"/>
+      <c r="AD207" s="5" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="AE207" s="5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AF207" s="5" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
       <c r="AG207" s="5" t="inlineStr"/>
       <c r="AH207" s="5" t="inlineStr"/>
-      <c r="AI207" s="5" t="inlineStr"/>
+      <c r="AI207" s="5" t="n">
+        <v>59.11691541835818</v>
+      </c>
       <c r="AJ207" s="5" t="inlineStr"/>
-      <c r="AK207" s="5" t="inlineStr"/>
+      <c r="AK207" s="5" t="n">
+        <v>-1.4</v>
+      </c>
       <c r="AL207" s="5" t="inlineStr"/>
-      <c r="AM207" s="5" t="inlineStr"/>
-      <c r="AN207" s="5" t="inlineStr"/>
-      <c r="AO207" s="5" t="inlineStr"/>
-      <c r="AP207" s="5" t="inlineStr"/>
-      <c r="AQ207" s="5" t="inlineStr"/>
-      <c r="AR207" s="5" t="inlineStr"/>
-      <c r="AS207" s="5" t="inlineStr"/>
-      <c r="AT207" s="5" t="inlineStr"/>
-      <c r="AU207" s="5" t="inlineStr"/>
-      <c r="AV207" s="5" t="inlineStr"/>
-      <c r="AW207" s="5" t="inlineStr"/>
+      <c r="AM207" s="5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AN207" s="5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AO207" s="5" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="AP207" s="5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AQ207" s="5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AR207" s="5" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="AS207" s="5" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="AT207" s="5" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="AU207" s="5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AV207" s="5" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="AW207" s="5" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
       <c r="AX207" s="5" t="inlineStr"/>
       <c r="AY207" s="5" t="inlineStr"/>
       <c r="AZ207" s="5" t="inlineStr"/>
@@ -43418,12 +43490,12 @@
       <c r="B208" s="3" t="inlineStr"/>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Nikola Jokić</t>
+          <t>Tim Hardaway</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G-F</t>
         </is>
       </c>
       <c r="E208" s="3" t="inlineStr">
@@ -43443,12 +43515,12 @@
       </c>
       <c r="H208" s="3" t="inlineStr">
         <is>
-          <t>Assists</t>
+          <t>Points</t>
         </is>
       </c>
       <c r="I208" s="3" t="inlineStr">
         <is>
-          <t>Goblin</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="J208" s="3" t="inlineStr">
@@ -43456,9 +43528,9 @@
           <t>2.5</t>
         </is>
       </c>
-      <c r="K208" s="4" t="inlineStr">
-        <is>
-          <t>OVER</t>
+      <c r="K208" s="6" t="inlineStr">
+        <is>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="L208" s="3" t="inlineStr"/>
@@ -43467,7 +43539,7 @@
         <v>0</v>
       </c>
       <c r="O208" s="3" t="n">
-        <v>0.8423</v>
+        <v>0.8335</v>
       </c>
       <c r="P208" s="3" t="inlineStr"/>
       <c r="Q208" s="3" t="inlineStr"/>
@@ -43587,7 +43659,7 @@
       </c>
       <c r="H209" s="5" t="inlineStr">
         <is>
-          <t>Rebounds</t>
+          <t>Assists</t>
         </is>
       </c>
       <c r="I209" s="5" t="inlineStr">
@@ -43611,7 +43683,7 @@
         <v>0</v>
       </c>
       <c r="O209" s="5" t="n">
-        <v>0.8525</v>
+        <v>0.8423</v>
       </c>
       <c r="P209" s="5" t="inlineStr"/>
       <c r="Q209" s="5" t="inlineStr"/>
@@ -43706,12 +43778,12 @@
       <c r="B210" s="3" t="inlineStr"/>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Tim Hardaway</t>
+          <t>Nikola Jokić</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
-          <t>G-F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E210" s="3" t="inlineStr">
@@ -43731,7 +43803,7 @@
       </c>
       <c r="H210" s="3" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>Rebounds</t>
         </is>
       </c>
       <c r="I210" s="3" t="inlineStr">
@@ -43741,7 +43813,7 @@
       </c>
       <c r="J210" s="3" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="K210" s="4" t="inlineStr">
@@ -43755,7 +43827,7 @@
         <v>0</v>
       </c>
       <c r="O210" s="3" t="n">
-        <v>0.8956</v>
+        <v>0.8525</v>
       </c>
       <c r="P210" s="3" t="inlineStr"/>
       <c r="Q210" s="3" t="inlineStr"/>
@@ -43875,17 +43947,17 @@
       </c>
       <c r="H211" s="5" t="inlineStr">
         <is>
-          <t>Assists</t>
+          <t>Points</t>
         </is>
       </c>
       <c r="I211" s="5" t="inlineStr">
         <is>
-          <t>Demon</t>
+          <t>Goblin</t>
         </is>
       </c>
       <c r="J211" s="5" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="K211" s="4" t="inlineStr">
@@ -43899,7 +43971,7 @@
         <v>0</v>
       </c>
       <c r="O211" s="5" t="n">
-        <v>0.72</v>
+        <v>0.8956</v>
       </c>
       <c r="P211" s="5" t="inlineStr"/>
       <c r="Q211" s="5" t="inlineStr"/>
@@ -43980,6 +44052,150 @@
         </is>
       </c>
       <c r="BJ211" s="5" t="inlineStr">
+        <is>
+          <t>No spread data: 0.97x default</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr"/>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>Tim Hardaway</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="inlineStr">
+        <is>
+          <t>G-F</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>DEN</t>
+        </is>
+      </c>
+      <c r="F212" s="3" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30 21:30:00-04:00</t>
+        </is>
+      </c>
+      <c r="H212" s="3" t="inlineStr">
+        <is>
+          <t>Assists</t>
+        </is>
+      </c>
+      <c r="I212" s="3" t="inlineStr">
+        <is>
+          <t>Demon</t>
+        </is>
+      </c>
+      <c r="J212" s="3" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="K212" s="4" t="inlineStr">
+        <is>
+          <t>OVER</t>
+        </is>
+      </c>
+      <c r="L212" s="3" t="inlineStr"/>
+      <c r="M212" s="3" t="inlineStr"/>
+      <c r="N212" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O212" s="3" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="P212" s="3" t="inlineStr"/>
+      <c r="Q212" s="3" t="inlineStr"/>
+      <c r="R212" s="3" t="inlineStr"/>
+      <c r="S212" s="3" t="inlineStr"/>
+      <c r="T212" s="3" t="inlineStr"/>
+      <c r="U212" s="3" t="inlineStr"/>
+      <c r="V212" s="3" t="inlineStr"/>
+      <c r="W212" s="3" t="inlineStr"/>
+      <c r="X212" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="Y212" s="3" t="inlineStr">
+        <is>
+          <t>Above Avg</t>
+        </is>
+      </c>
+      <c r="Z212" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="AA212" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="AB212" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="AC212" s="3" t="inlineStr">
+        <is>
+          <t>NO_PROJECTION_OR_LINE</t>
+        </is>
+      </c>
+      <c r="AD212" s="3" t="inlineStr"/>
+      <c r="AE212" s="3" t="inlineStr"/>
+      <c r="AF212" s="3" t="inlineStr"/>
+      <c r="AG212" s="3" t="inlineStr"/>
+      <c r="AH212" s="3" t="inlineStr"/>
+      <c r="AI212" s="3" t="inlineStr"/>
+      <c r="AJ212" s="3" t="inlineStr"/>
+      <c r="AK212" s="3" t="inlineStr"/>
+      <c r="AL212" s="3" t="inlineStr"/>
+      <c r="AM212" s="3" t="inlineStr"/>
+      <c r="AN212" s="3" t="inlineStr"/>
+      <c r="AO212" s="3" t="inlineStr"/>
+      <c r="AP212" s="3" t="inlineStr"/>
+      <c r="AQ212" s="3" t="inlineStr"/>
+      <c r="AR212" s="3" t="inlineStr"/>
+      <c r="AS212" s="3" t="inlineStr"/>
+      <c r="AT212" s="3" t="inlineStr"/>
+      <c r="AU212" s="3" t="inlineStr"/>
+      <c r="AV212" s="3" t="inlineStr"/>
+      <c r="AW212" s="3" t="inlineStr"/>
+      <c r="AX212" s="3" t="inlineStr"/>
+      <c r="AY212" s="3" t="inlineStr"/>
+      <c r="AZ212" s="3" t="inlineStr"/>
+      <c r="BA212" s="3" t="inlineStr"/>
+      <c r="BB212" s="3" t="inlineStr"/>
+      <c r="BC212" s="3" t="inlineStr"/>
+      <c r="BD212" s="3" t="inlineStr"/>
+      <c r="BE212" s="3" t="inlineStr"/>
+      <c r="BF212" s="3" t="inlineStr"/>
+      <c r="BG212" s="3" t="inlineStr"/>
+      <c r="BH212" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI212" s="3" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="BJ212" s="3" t="inlineStr">
         <is>
           <t>No spread data: 0.97x default</t>
         </is>
@@ -70558,7 +70774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ93"/>
+  <dimension ref="A1:BJ94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -82166,7 +82382,7 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
@@ -87938,24 +88154,24 @@
       <c r="B89" s="5" t="inlineStr"/>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Tim Hardaway</t>
+          <t>Rudy Gobert</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>G-F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
           <t>DEN</t>
         </is>
       </c>
-      <c r="F89" s="5" t="inlineStr">
-        <is>
-          <t>MIN</t>
-        </is>
-      </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
           <t>2026-04-30 21:30:00-04:00</t>
@@ -87981,30 +88197,46 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="L89" s="5" t="inlineStr"/>
-      <c r="M89" s="5" t="inlineStr"/>
+      <c r="L89" s="5" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="M89" s="5" t="n">
+        <v>0.2</v>
+      </c>
       <c r="N89" s="5" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="O89" s="5" t="n">
-        <v>0.8335</v>
+        <v>0.8636</v>
       </c>
       <c r="P89" s="5" t="inlineStr"/>
       <c r="Q89" s="5" t="inlineStr"/>
-      <c r="R89" s="5" t="inlineStr"/>
-      <c r="S89" s="5" t="inlineStr"/>
-      <c r="T89" s="5" t="inlineStr"/>
-      <c r="U89" s="5" t="inlineStr"/>
-      <c r="V89" s="5" t="inlineStr"/>
-      <c r="W89" s="5" t="inlineStr"/>
+      <c r="R89" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="S89" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="T89" s="5" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="U89" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="V89" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="W89" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="X89" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>21</t>
         </is>
       </c>
       <c r="Y89" s="5" t="inlineStr">
         <is>
-          <t>Above Avg</t>
+          <t>Avg</t>
         </is>
       </c>
       <c r="Z89" s="5" t="inlineStr">
@@ -88019,34 +88251,90 @@
       </c>
       <c r="AB89" s="5" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="AC89" s="5" t="inlineStr">
-        <is>
-          <t>NO_PROJECTION_OR_LINE</t>
-        </is>
-      </c>
-      <c r="AD89" s="5" t="inlineStr"/>
-      <c r="AE89" s="5" t="inlineStr"/>
-      <c r="AF89" s="5" t="inlineStr"/>
+          <t>SUPPORT</t>
+        </is>
+      </c>
+      <c r="AC89" s="5" t="inlineStr"/>
+      <c r="AD89" s="5" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="AE89" s="5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AF89" s="5" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
       <c r="AG89" s="5" t="inlineStr"/>
       <c r="AH89" s="5" t="inlineStr"/>
-      <c r="AI89" s="5" t="inlineStr"/>
+      <c r="AI89" s="5" t="n">
+        <v>59.11691541835818</v>
+      </c>
       <c r="AJ89" s="5" t="inlineStr"/>
-      <c r="AK89" s="5" t="inlineStr"/>
+      <c r="AK89" s="5" t="n">
+        <v>-1.4</v>
+      </c>
       <c r="AL89" s="5" t="inlineStr"/>
-      <c r="AM89" s="5" t="inlineStr"/>
-      <c r="AN89" s="5" t="inlineStr"/>
-      <c r="AO89" s="5" t="inlineStr"/>
-      <c r="AP89" s="5" t="inlineStr"/>
-      <c r="AQ89" s="5" t="inlineStr"/>
-      <c r="AR89" s="5" t="inlineStr"/>
-      <c r="AS89" s="5" t="inlineStr"/>
-      <c r="AT89" s="5" t="inlineStr"/>
-      <c r="AU89" s="5" t="inlineStr"/>
-      <c r="AV89" s="5" t="inlineStr"/>
-      <c r="AW89" s="5" t="inlineStr"/>
+      <c r="AM89" s="5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AN89" s="5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AO89" s="5" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="AP89" s="5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AQ89" s="5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AR89" s="5" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="AS89" s="5" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="AT89" s="5" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="AU89" s="5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AV89" s="5" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="AW89" s="5" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
       <c r="AX89" s="5" t="inlineStr"/>
       <c r="AY89" s="5" t="inlineStr"/>
       <c r="AZ89" s="5" t="inlineStr"/>
@@ -88082,12 +88370,12 @@
       <c r="B90" s="3" t="inlineStr"/>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Nikola Jokić</t>
+          <t>Tim Hardaway</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G-F</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
@@ -88107,12 +88395,12 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>Assists</t>
+          <t>Points</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>Goblin</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
@@ -88120,9 +88408,9 @@
           <t>2.5</t>
         </is>
       </c>
-      <c r="K90" s="4" t="inlineStr">
-        <is>
-          <t>OVER</t>
+      <c r="K90" s="6" t="inlineStr">
+        <is>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="L90" s="3" t="inlineStr"/>
@@ -88131,7 +88419,7 @@
         <v>0</v>
       </c>
       <c r="O90" s="3" t="n">
-        <v>0.8423</v>
+        <v>0.8335</v>
       </c>
       <c r="P90" s="3" t="inlineStr"/>
       <c r="Q90" s="3" t="inlineStr"/>
@@ -88251,7 +88539,7 @@
       </c>
       <c r="H91" s="5" t="inlineStr">
         <is>
-          <t>Rebounds</t>
+          <t>Assists</t>
         </is>
       </c>
       <c r="I91" s="5" t="inlineStr">
@@ -88275,7 +88563,7 @@
         <v>0</v>
       </c>
       <c r="O91" s="5" t="n">
-        <v>0.8525</v>
+        <v>0.8423</v>
       </c>
       <c r="P91" s="5" t="inlineStr"/>
       <c r="Q91" s="5" t="inlineStr"/>
@@ -88370,12 +88658,12 @@
       <c r="B92" s="3" t="inlineStr"/>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Tim Hardaway</t>
+          <t>Nikola Jokić</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>G-F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
@@ -88395,7 +88683,7 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>Rebounds</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
@@ -88405,7 +88693,7 @@
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="K92" s="4" t="inlineStr">
@@ -88419,7 +88707,7 @@
         <v>0</v>
       </c>
       <c r="O92" s="3" t="n">
-        <v>0.8956</v>
+        <v>0.8525</v>
       </c>
       <c r="P92" s="3" t="inlineStr"/>
       <c r="Q92" s="3" t="inlineStr"/>
@@ -88539,17 +88827,17 @@
       </c>
       <c r="H93" s="5" t="inlineStr">
         <is>
-          <t>Assists</t>
+          <t>Points</t>
         </is>
       </c>
       <c r="I93" s="5" t="inlineStr">
         <is>
-          <t>Demon</t>
+          <t>Goblin</t>
         </is>
       </c>
       <c r="J93" s="5" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="K93" s="4" t="inlineStr">
@@ -88563,7 +88851,7 @@
         <v>0</v>
       </c>
       <c r="O93" s="5" t="n">
-        <v>0.72</v>
+        <v>0.8956</v>
       </c>
       <c r="P93" s="5" t="inlineStr"/>
       <c r="Q93" s="5" t="inlineStr"/>
@@ -88649,6 +88937,150 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr"/>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Tim Hardaway</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>G-F</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>DEN</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30 21:30:00-04:00</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>Assists</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>Demon</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="K94" s="4" t="inlineStr">
+        <is>
+          <t>OVER</t>
+        </is>
+      </c>
+      <c r="L94" s="3" t="inlineStr"/>
+      <c r="M94" s="3" t="inlineStr"/>
+      <c r="N94" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" s="3" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="P94" s="3" t="inlineStr"/>
+      <c r="Q94" s="3" t="inlineStr"/>
+      <c r="R94" s="3" t="inlineStr"/>
+      <c r="S94" s="3" t="inlineStr"/>
+      <c r="T94" s="3" t="inlineStr"/>
+      <c r="U94" s="3" t="inlineStr"/>
+      <c r="V94" s="3" t="inlineStr"/>
+      <c r="W94" s="3" t="inlineStr"/>
+      <c r="X94" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="Y94" s="3" t="inlineStr">
+        <is>
+          <t>Above Avg</t>
+        </is>
+      </c>
+      <c r="Z94" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="AA94" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="AB94" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="AC94" s="3" t="inlineStr">
+        <is>
+          <t>NO_PROJECTION_OR_LINE</t>
+        </is>
+      </c>
+      <c r="AD94" s="3" t="inlineStr"/>
+      <c r="AE94" s="3" t="inlineStr"/>
+      <c r="AF94" s="3" t="inlineStr"/>
+      <c r="AG94" s="3" t="inlineStr"/>
+      <c r="AH94" s="3" t="inlineStr"/>
+      <c r="AI94" s="3" t="inlineStr"/>
+      <c r="AJ94" s="3" t="inlineStr"/>
+      <c r="AK94" s="3" t="inlineStr"/>
+      <c r="AL94" s="3" t="inlineStr"/>
+      <c r="AM94" s="3" t="inlineStr"/>
+      <c r="AN94" s="3" t="inlineStr"/>
+      <c r="AO94" s="3" t="inlineStr"/>
+      <c r="AP94" s="3" t="inlineStr"/>
+      <c r="AQ94" s="3" t="inlineStr"/>
+      <c r="AR94" s="3" t="inlineStr"/>
+      <c r="AS94" s="3" t="inlineStr"/>
+      <c r="AT94" s="3" t="inlineStr"/>
+      <c r="AU94" s="3" t="inlineStr"/>
+      <c r="AV94" s="3" t="inlineStr"/>
+      <c r="AW94" s="3" t="inlineStr"/>
+      <c r="AX94" s="3" t="inlineStr"/>
+      <c r="AY94" s="3" t="inlineStr"/>
+      <c r="AZ94" s="3" t="inlineStr"/>
+      <c r="BA94" s="3" t="inlineStr"/>
+      <c r="BB94" s="3" t="inlineStr"/>
+      <c r="BC94" s="3" t="inlineStr"/>
+      <c r="BD94" s="3" t="inlineStr"/>
+      <c r="BE94" s="3" t="inlineStr"/>
+      <c r="BF94" s="3" t="inlineStr"/>
+      <c r="BG94" s="3" t="inlineStr"/>
+      <c r="BH94" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI94" s="3" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="BJ94" s="3" t="inlineStr">
+        <is>
+          <t>No spread data: 0.97x default</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:BJ1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>